<commit_message>
feat: replace free run tag with penalty focus
</commit_message>
<xml_diff>
--- a/output/test-config/level-tags/LevelTagCfg.xlsx
+++ b/output/test-config/level-tags/LevelTagCfg.xlsx
@@ -513,6 +513,11 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8"/>
     <row r="9">
       <c r="A9" t="n">
         <v>1</v>
@@ -528,12 +533,12 @@
       </c>
       <c r="E9" t="inlineStr">
         <is>
-          <t>tutorial, free_run</t>
+          <t>tutorial, penalty_focus</t>
         </is>
       </c>
       <c r="F9" t="inlineStr">
         <is>
-          <t>恢复:短局免票,给玩家重新进入心流</t>
+          <t>恢复:短局点球确定性,给玩家重新进入心流</t>
         </is>
       </c>
     </row>
@@ -740,12 +745,12 @@
       </c>
       <c r="E19" t="inlineStr">
         <is>
-          <t>short_match, free_run</t>
+          <t>short_match, penalty_focus</t>
         </is>
       </c>
       <c r="F19" t="inlineStr">
         <is>
-          <t>恢复:短局免票,给玩家重新进入心流</t>
+          <t>恢复:短局点球确定性,给玩家重新进入心流</t>
         </is>
       </c>
     </row>
@@ -948,12 +953,12 @@
       </c>
       <c r="E29" t="inlineStr">
         <is>
-          <t>short_match, free_run</t>
+          <t>short_match, penalty_focus</t>
         </is>
       </c>
       <c r="F29" t="inlineStr">
         <is>
-          <t>恢复:短局免票,给玩家重新进入心流</t>
+          <t>恢复:短局点球确定性,给玩家重新进入心流</t>
         </is>
       </c>
     </row>
@@ -1160,12 +1165,12 @@
       </c>
       <c r="E39" t="inlineStr">
         <is>
-          <t>short_match, free_run</t>
+          <t>short_match, penalty_focus</t>
         </is>
       </c>
       <c r="F39" t="inlineStr">
         <is>
-          <t>恢复:短局免票,给玩家重新进入心流</t>
+          <t>恢复:短局点球确定性,给玩家重新进入心流</t>
         </is>
       </c>
     </row>
@@ -1368,12 +1373,12 @@
       </c>
       <c r="E49" t="inlineStr">
         <is>
-          <t>short_match, free_run</t>
+          <t>short_match, penalty_focus</t>
         </is>
       </c>
       <c r="F49" t="inlineStr">
         <is>
-          <t>恢复:短局免票,给玩家重新进入心流</t>
+          <t>恢复:短局点球确定性,给玩家重新进入心流</t>
         </is>
       </c>
     </row>
@@ -1584,12 +1589,12 @@
       </c>
       <c r="E59" t="inlineStr">
         <is>
-          <t>short_match, free_run</t>
+          <t>short_match, penalty_focus</t>
         </is>
       </c>
       <c r="F59" t="inlineStr">
         <is>
-          <t>恢复:短局免票,给玩家重新进入心流</t>
+          <t>恢复:短局点球确定性,给玩家重新进入心流</t>
         </is>
       </c>
     </row>
@@ -1796,12 +1801,12 @@
       </c>
       <c r="E69" t="inlineStr">
         <is>
-          <t>short_match, free_run</t>
+          <t>short_match, penalty_focus</t>
         </is>
       </c>
       <c r="F69" t="inlineStr">
         <is>
-          <t>恢复:短局免票,给玩家重新进入心流</t>
+          <t>恢复:短局点球确定性,给玩家重新进入心流</t>
         </is>
       </c>
     </row>
@@ -2012,12 +2017,12 @@
       </c>
       <c r="E79" t="inlineStr">
         <is>
-          <t>short_match, free_run</t>
+          <t>short_match, penalty_focus</t>
         </is>
       </c>
       <c r="F79" t="inlineStr">
         <is>
-          <t>恢复:短局免票,给玩家重新进入心流</t>
+          <t>恢复:短局点球确定性,给玩家重新进入心流</t>
         </is>
       </c>
     </row>
@@ -2224,12 +2229,12 @@
       </c>
       <c r="E89" t="inlineStr">
         <is>
-          <t>short_match, free_run</t>
+          <t>short_match, penalty_focus</t>
         </is>
       </c>
       <c r="F89" t="inlineStr">
         <is>
-          <t>恢复:短局免票,给玩家重新进入心流</t>
+          <t>恢复:短局点球确定性,给玩家重新进入心流</t>
         </is>
       </c>
     </row>
@@ -2440,12 +2445,12 @@
       </c>
       <c r="E99" t="inlineStr">
         <is>
-          <t>short_match, free_run</t>
+          <t>short_match, penalty_focus</t>
         </is>
       </c>
       <c r="F99" t="inlineStr">
         <is>
-          <t>恢复:短局免票,给玩家重新进入心流</t>
+          <t>恢复:短局点球确定性,给玩家重新进入心流</t>
         </is>
       </c>
     </row>
@@ -11977,6 +11982,11 @@
         </is>
       </c>
     </row>
+    <row r="4"/>
+    <row r="5"/>
+    <row r="6"/>
+    <row r="7"/>
+    <row r="8"/>
     <row r="9">
       <c r="A9" t="inlineStr">
         <is>
@@ -12075,129 +12085,134 @@
     <row r="14">
       <c r="A14" t="inlineStr">
         <is>
-          <t>free_run</t>
+          <t>gk_test</t>
         </is>
       </c>
       <c r="B14" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>slice</t>
         </is>
       </c>
       <c r="D14" t="inlineStr">
         <is>
-          <t>门票消耗 0</t>
+          <t>末位强制 goalkeep v2</t>
         </is>
       </c>
     </row>
     <row r="15">
       <c r="A15" t="inlineStr">
         <is>
-          <t>gk_test</t>
+          <t>hard_plus</t>
         </is>
       </c>
       <c r="B15" t="inlineStr">
         <is>
-          <t>slice</t>
+          <t>ai</t>
+        </is>
+      </c>
+      <c r="C15" t="inlineStr">
+        <is>
+          <t>difficulty</t>
         </is>
       </c>
       <c r="D15" t="inlineStr">
         <is>
-          <t>末位强制 goalkeep v2</t>
+          <t>AiProfile +1 + OpponentStar +1</t>
         </is>
       </c>
     </row>
     <row r="16">
       <c r="A16" t="inlineStr">
         <is>
-          <t>hard_plus</t>
+          <t>lenient</t>
         </is>
       </c>
       <c r="B16" t="inlineStr">
         <is>
-          <t>ai</t>
+          <t>level</t>
         </is>
       </c>
       <c r="C16" t="inlineStr">
         <is>
-          <t>difficulty</t>
+          <t>threshold</t>
         </is>
       </c>
       <c r="D16" t="inlineStr">
         <is>
-          <t>AiProfile +1 + OpponentStar +1</t>
+          <t>胜阈值降至 40%</t>
         </is>
       </c>
     </row>
     <row r="17">
       <c r="A17" t="inlineStr">
         <is>
-          <t>lenient</t>
+          <t>long_match</t>
         </is>
       </c>
       <c r="B17" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>slice</t>
         </is>
       </c>
       <c r="C17" t="inlineStr">
         <is>
-          <t>threshold</t>
+          <t>length</t>
         </is>
       </c>
       <c r="D17" t="inlineStr">
         <is>
-          <t>胜阈值降至 40%</t>
+          <t>切片数 +1(上限 5)</t>
         </is>
       </c>
     </row>
     <row r="18">
       <c r="A18" t="inlineStr">
         <is>
-          <t>long_match</t>
+          <t>must_win</t>
         </is>
       </c>
       <c r="B18" t="inlineStr">
         <is>
-          <t>slice</t>
+          <t>level</t>
         </is>
       </c>
       <c r="C18" t="inlineStr">
         <is>
-          <t>length</t>
+          <t>threshold</t>
         </is>
       </c>
       <c r="D18" t="inlineStr">
         <is>
-          <t>切片数 +1(上限 5)</t>
+          <t>切片全胜才能赢</t>
         </is>
       </c>
     </row>
     <row r="19">
       <c r="A19" t="inlineStr">
         <is>
-          <t>must_win</t>
+          <t>narrow_angle</t>
         </is>
       </c>
       <c r="B19" t="inlineStr">
         <is>
-          <t>level</t>
+          <t>ai</t>
         </is>
       </c>
       <c r="C19" t="inlineStr">
         <is>
-          <t>threshold</t>
+          <t>modifier</t>
         </is>
       </c>
       <c r="D19" t="inlineStr">
         <is>
-          <t>切片全胜才能赢</t>
+          <t>ModifierID 强制 4006</t>
         </is>
       </c>
     </row>
     <row r="20">
       <c r="A20" t="inlineStr">
         <is>
-          <t>narrow_angle</t>
+          <t>no_modifier</t>
         </is>
       </c>
       <c r="B20" t="inlineStr">
@@ -12212,29 +12227,24 @@
       </c>
       <c r="D20" t="inlineStr">
         <is>
-          <t>ModifierID 强制 4006</t>
+          <t>ModifierID 强制 0</t>
         </is>
       </c>
     </row>
     <row r="21">
       <c r="A21" t="inlineStr">
         <is>
-          <t>no_modifier</t>
+          <t>penalty_focus</t>
         </is>
       </c>
       <c r="B21" t="inlineStr">
         <is>
-          <t>ai</t>
-        </is>
-      </c>
-      <c r="C21" t="inlineStr">
-        <is>
-          <t>modifier</t>
+          <t>slice</t>
         </is>
       </c>
       <c r="D21" t="inlineStr">
         <is>
-          <t>ModifierID 强制 0</t>
+          <t>保证至少 1 penalty 切片</t>
         </is>
       </c>
     </row>

</xml_diff>